<commit_message>
Update trade log, recommendations, and news corpus; add CLAUDE.md
Records today's trading session (closed the initial two trades, opened
four new call/put spreads across the 9/30 and 10/16 expiries) and the
screener runs behind them. Adds two more days of fetched news to the
corpus archive, plus the project's CLAUDE.md instructions file, which
had never been committed.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/portfolio/trade_log.xlsx
+++ b/data/portfolio/trade_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N5"/>
+  <dimension ref="A1:N13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -533,9 +533,17 @@
       <c r="J2" t="n">
         <v>37.85</v>
       </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="L2" t="n">
+        <v>54.8</v>
+      </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>CLOSED</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -589,9 +597,17 @@
       <c r="J3" t="n">
         <v>27.8</v>
       </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="L3" t="n">
+        <v>39.5</v>
+      </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>CLOSED</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -645,9 +661,17 @@
       <c r="J4" t="n">
         <v>14.5</v>
       </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="L4" t="n">
+        <v>4.9</v>
+      </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>CLOSED</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -701,14 +725,440 @@
       <c r="J5" t="n">
         <v>5.6</v>
       </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="L5" t="n">
+        <v>1.73</v>
+      </c>
       <c r="M5" t="inlineStr">
         <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>manual add (user override, not picker-vetted). User-specified call spread per Fed-hike sentiment view</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>SPX-CS-20260930-7950x8050</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>call spread</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>7950</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>20</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
           <t>OPEN</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>manual add (user override, not picker-vetted). User-specified call spread per Fed-hike sentiment view</t>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>SPX-CS-20260930-7950x8050</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>call spread</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>8050</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>20</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="J7" t="n">
+        <v>3.95</v>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>SPX-PS-20260930-7400x7300</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>put spread</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>7400</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
+        <v>20</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="J8" t="n">
+        <v>35.75</v>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>SPX-PS-20260930-7400x7300</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>put spread</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>7300</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>20</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="J9" t="n">
+        <v>25.85</v>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>SPX-PS-20261016-7400x7300</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>put spread</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>7400</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="H10" t="n">
+        <v>20</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="J10" t="n">
+        <v>56.85</v>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>SPX-PS-20261016-7400x7300</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>put spread</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>7300</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="H11" t="n">
+        <v>20</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="J11" t="n">
+        <v>44.3</v>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>SPX-CS-20261016-8000x8100</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>call spread</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>8000</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="H12" t="n">
+        <v>20</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="J12" t="n">
+        <v>25.25</v>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>manual add (user override, not picker-vetted). user-specified call spread</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>SPX-CS-20261016-8000x8100</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>call spread</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>8100</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="H13" t="n">
+        <v>20</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="J13" t="n">
+        <v>11.85</v>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>manual add (user override, not picker-vetted). user-specified call spread</t>
         </is>
       </c>
     </row>

</xml_diff>